<commit_message>
vault backup: 2026-08-02 00:28:25
</commit_message>
<xml_diff>
--- a/Codex/projects/考研英语外刊精读/articles/The two Cambridges/anki/anki.xlsx
+++ b/Codex/projects/考研英语外刊精读/articles/The two Cambridges/anki/anki.xlsx
@@ -41,12 +41,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：浸润于，充满。&lt;br&gt;&lt;b&gt;本义&lt;/b&gt;：steep 可指把东西浸泡在液体里。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：某地、组织或领域长期浸润在某种传统、文化、精神或氛围中。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：文雅、书面，比 be full of 更有历史厚度。</t>
+          <t>字面含义：浸润于；充满；深深带有
+考研核心考点：文化/城市/传统/创新类高分表达
+词汇拆解：steep 本义是“浸泡”；be steeped in = be deeply filled with/strongly influenced by
+熟词辟义/一词多义：steep 不只是“陡峭的”，作动词可指“浸泡”，引申为被某种氛围长期浸润。
+语气色彩：文雅、书面、带历史厚度</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Cambridge is steeped in innovation. 作者不是说剑桥“有创新”，而是说创新像传统一样渗透其中。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：创新不是偶然事件，而是长期积累出的城市气质。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：A great university should be steeped in curiosity and intellectual discipline.&lt;br&gt;&lt;b&gt;例句2 文化&lt;/b&gt;：A city steeped in tradition can still embrace modern technology.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：Contemporary society is steeped in digital innovation, but it also needs ethical reflection.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育学习、传统文化、科技创新、城市发展。</t>
+          <t>文章语境：文章说 Cambridge is steeped in innovation，强调创新像传统一样渗透城市。
+暗示意思/政治意味/诙谐意味：暗示创新不是偶然，而是长期制度、大学和资本共同塑造的城市气质。
+特殊考查方式：写作替换 be full of；翻译题考抽象义。
+答题技巧：看到 be steeped in + 抽象名词，译为“深受……浸润/充满……氛围”。
+同义替换/错误选项信号：be full of; be immersed in; be saturated with; be rich in
+多场景例句：be steeped in innovation；a city steeped in tradition；a campus steeped in intellectual curiosity
+其他可用地方：文化、教育、科技创新、城市发展</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -58,17 +68,28 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>namesake</t>
+          <t>have the edge in</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：同名者，同名地。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：名字相同但身份、地位、发展路径可能不同的人或地方。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：新闻和文化类文章常用，用来引出比较或历史渊源。</t>
+          <t>字面含义：在……方面占优势
+考研核心考点：比较类阅读和作文高频
+词汇拆解：edge = 边缘；引申为优势；have the edge in/over = have an advantage in/over
+熟词辟义/一词多义：edge 不只是“边缘”，外刊常指竞争优势。
+语气色彩：正式中性，竞争语境明显</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：American namesake 指美国马萨诸塞州剑桥，与英国剑桥同名。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：同名不只是巧合，而是历史、教育和文化联系。&lt;br&gt;&lt;b&gt;例句1 文化&lt;/b&gt;：The American city shares both its name and academic ambition with its British namesake.&lt;br&gt;&lt;b&gt;例句2 品牌&lt;/b&gt;：A product may borrow the prestige of its famous namesake, but it must prove its own value.&lt;br&gt;&lt;b&gt;例句3 写作&lt;/b&gt;：Cultural influence can travel across borders and reappear in a distant namesake.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：文化交流、历史渊源、城市比较、品牌命名。</t>
+          <t>文章语境：文章比较英美两个 Cambridge 在商业化、资本、科研等方面谁更有优势。
+暗示意思/政治意味/诙谐意味：暗示优势不是绝对全面，而是在某个维度上领先。
+特殊考查方式：细节/态度题会用 advantage/lead 替换。
+答题技巧：注意介词：have the edge in + 领域；have the edge over + 对手。
+同义替换/错误选项信号：have an advantage in; lead in; outperform in; be ahead in
+多场景例句：have the edge in commercialising research；have the edge over rivals；gain an edge in the job market
+其他可用地方：经济竞争、教育优势、职场发展
+归一化合并：本卡覆盖这些变体：have the edge</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -80,17 +101,28 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>not so much A as B</t>
+          <t>commercialise research</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：与其说 A，不如说 B。&lt;br&gt;&lt;b&gt;语法&lt;/b&gt;：重点不是完全否定 A，而是强调 B 更准确。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：高级转折，适合纠正表面理解。</t>
+          <t>字面含义：将研究商业化
+考研核心考点：科技创新与经济转化核心搭配
+词汇拆解：commercialise = make commercially usable/profitable；research = 科研成果
+熟词辟义/一词多义：research 不只指论文，也可指可转化的技术成果。
+语气色彩：正式、中性偏经济</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：American Cambridge has not so much imitated its British cousin as surpassed it. 作者强调美国剑桥不只是模仿，而是超越。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：美国创新生态已经从继承者变成领先者。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Online learning has not so much replaced classrooms as expanded what education can be.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：AI has not so much removed human judgment as made it more important.&lt;br&gt;&lt;b&gt;例句3 职场&lt;/b&gt;：A good job has not so much given me comfort as forced me to grow.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技双刃剑、教育改革、个人成长、社会变化。</t>
+          <t>文章语境：文章比较两地把大学科研转化为企业和产品的能力。
+暗示意思/政治意味/诙谐意味：暗示真正的创新不止在实验室，还要走向市场。
+特殊考查方式：细节题常问 university research 如何变成 companies/products。
+答题技巧：commercialise 后面常接 research, technology, discovery；不要译成“商业研究”。
+同义替换/错误选项信号：turn research into products; bring discoveries to market; translate research into business
+多场景例句：commercialise university research；commercialise medical discoveries；turn basic research into marketable products
+其他可用地方：科技创新、产学研、职场创业
+归一化合并：本卡覆盖这些变体：commercialise research</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -102,17 +134,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>mirror images</t>
+          <t>innovation cluster</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：镜像，彼此像镜子里的对应物。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：表面相似，但方向、问题或结构相反。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：形象对比，适合写议论文结构。</t>
+          <t>字面含义：创新集群
+考研核心考点：科技经济类主题词
+词汇拆解：innovation = 创新；cluster = 聚集/集群
+熟词辟义/一词多义：cluster 不只是“簇”，经济地理中指企业、大学、人才和资本集中区。
+语气色彩：正式、经济地理语体</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：The two Cambridges are mirror images: on the surface almost identical, but with opposite problems. 两地都强创新，但短板相反。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：文章不是简单排名，而是结构性比较。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Urban and rural schools can be mirror images: one has resources but pressure, the other has freedom but fewer opportunities.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：Two platforms may be mirror images, sharing the same users but creating opposite social effects.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：Modern life often presents mirror images of progress: more convenience, but less patience.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：对比论证、城市发展、教育公平、科技影响。</t>
+          <t>文章语境：文章把两个 Cambridge 都看作大学、资本、公司密集互动的创新集群。
+暗示意思/政治意味/诙谐意味：暗示创新来自生态系统，不是单个天才或单所大学。
+特殊考查方式：主旨题可用 ecosystem/hub/network 替换。
+答题技巧：遇到 cluster 要想到“地理集中 + 网络效应”。
+同义替换/错误选项信号：innovation hub; tech cluster; entrepreneurial ecosystem
+多场景例句：an innovation cluster around a university；a biotech innovation cluster；build a regional innovation ecosystem
+其他可用地方：科技、经济、城市发展</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -124,17 +166,27 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>offset weaknesses</t>
+          <t>be constrained by</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：抵消弱点，弥补短板。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：offset 可作动词，表示用一方抵消另一方。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济、管理、合作语境常用。</t>
+          <t>字面含义：受……限制/约束
+考研核心考点：原因分析类高频被动结构
+词汇拆解：constrain = limit/restrict；be constrained by + 限制因素
+熟词辟义/一词多义：constraint 是“限制条件”，不是简单 difficulty。
+语气色彩：正式、中性偏负面</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：两个剑桥更紧密合作 to offset weaknesses。合作不是情怀，而是互补短板。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：真正有效的合作来自互补，而不只是相似。&lt;br&gt;&lt;b&gt;例句1 学习&lt;/b&gt;：Group study can offset individual weaknesses if members have different strengths.&lt;br&gt;&lt;b&gt;例句2 职场&lt;/b&gt;：A strong team offsets weaknesses through complementary skills.&lt;br&gt;&lt;b&gt;例句3 经济&lt;/b&gt;：Public investment can offset weaknesses in private capital markets.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：团队合作、教育学习、区域合作、经济政策。</t>
+          <t>文章语境：文章说英国剑桥的发展受空间、资本或城市条件约束。
+暗示意思/政治意味/诙谐意味：暗示潜力存在，但外部条件限制其释放。
+特殊考查方式：原因题常考 by 后面的限制因素。
+答题技巧：翻译时把被动转主动也可：X 限制了 Y。
+同义替换/错误选项信号：be limited by; be restricted by; be held back by
+多场景例句：be constrained by limited space；be constrained by old institutions；growth constrained by capital shortages
+其他可用地方：教育资源、城市发展、职场限制</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -146,17 +198,28 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>conjoined</t>
+          <t>be starved of capital and space</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：连接在一起的，结合的。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：关系越来越紧密，难以完全分开。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：比 connected 更强，带结构性绑定意味。</t>
+          <t>字面含义：缺乏资本和空间；资本和空间严重不足
+考研核心考点：starve 的抽象用法
+词汇拆解：starve = 挨饿；be starved of = be deprived of/lack badly
+熟词辟义/一词多义：starved 不只指食物匮乏，可指资源严重不足。
+语气色彩：形象、负面、外刊常用</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：The relationship is unequal, but increasingly conjoined. 两个剑桥不对等，但越来越相连。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：合作不是完全平等的联盟，而是互相依赖的结构。&lt;br&gt;&lt;b&gt;例句1 经济&lt;/b&gt;：Education and employment are increasingly conjoined in the modern economy.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：Technology and daily life have become deeply conjoined.&lt;br&gt;&lt;b&gt;例句3 写作&lt;/b&gt;：Personal freedom and social responsibility are conjoined rather than opposed.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技生活、教育就业、社会责任、国际合作。</t>
+          <t>文章语境：文章说英国剑桥 starved of capital and space，制约企业成长。
+暗示意思/政治意味/诙谐意味：暗示不是没有能力，而是缺钱、缺地、缺设施。
+特殊考查方式：词义题会考 starved of 的非字面义。
+答题技巧：看到 be starved of + 抽象资源，译为“严重缺乏……”。
+同义替换/错误选项信号：be short of; lack; be deprived of; suffer from a shortage of
+多场景例句：be starved of capital and space；schools starved of resources；start-ups starved of funding
+其他可用地方：教育公平、创业、城市资源
+归一化合并：本卡覆盖这些变体：be starved of</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -168,17 +231,27 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>innovation engine</t>
+          <t>proof of concept</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：创新引擎。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：持续产生新技术、新公司、新人才和新产业的系统。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济报道和政策文本常用。</t>
+          <t>字面含义：概念验证；可行性证明
+考研核心考点：科技/创业类核心术语
+词汇拆解：proof = 证明；concept = 概念；证明某想法可行
+熟词辟义/一词多义：proof 不只是“证据”，在科技商业中是早期可行性验证。
+语气色彩：技术商业语体</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：两个剑桥都是 efficient innovation engines。作者强调它们不是单个大学，而是能持续产出的系统。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：创新靠生态，不靠孤立天才。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Universities can become innovation engines when research is connected with society.&lt;br&gt;&lt;b&gt;例句2 城市&lt;/b&gt;：A city becomes an innovation engine when talent, capital and infrastructure interact.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：Education is the most reliable innovation engine for long-term national development.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育强国、科技创新、城市发展、经济转型。</t>
+          <t>文章语境：文章讨论科研成果从实验室到商业化时需要 proof of concept。
+暗示意思/政治意味/诙谐意味：暗示科学想法要先证明可做，才可能吸引资本。
+特殊考查方式：细节题常问 early-stage validation。
+答题技巧：不要译成“概念的证明”那么生硬，可译“概念验证”。
+同义替换/错误选项信号：feasibility test; early validation; prototype evidence
+多场景例句：provide proof of concept；fund proof-of-concept research；move from proof of concept to production
+其他可用地方：科技创新、创业、学习项目</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -190,17 +263,27 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>have the edge in</t>
+          <t>risk-averse</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：在某方面略占优势。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：比较时常用，通常不是绝对碾压，而是相对领先。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：have the edge in research / quality / speed / experience。</t>
+          <t>字面含义：厌恶风险的；避险的
+考研核心考点：经济/心理/政策态度词
+词汇拆解：risk = 风险；averse = 反感的；risk-averse = unwilling to take risks
+熟词辟义/一词多义：averse 常与 to 搭配；risk-averse 是合成形容词。
+语气色彩：正式、中性偏批评</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Britain's Cambridge may have the edge in research. 英国剑桥科研更强，但商业化不如波士顿。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：优势是局部的，不能推出整体更强。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Traditional classrooms still have the edge in discipline and face-to-face interaction.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：Small firms may have the edge in flexibility, while large firms have more resources.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：A country can have the edge in research but still lag behind in application.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：对比论证、教育方式、科技竞争、职场能力。</t>
+          <t>文章语境：文章用它描述资本或机构不愿承担早期创新风险。
+暗示意思/政治意味/诙谐意味：暗示过度保守会拖慢创新商业化。
+特殊考查方式：态度题常考作者是否批评保守资本。
+答题技巧：和 cautious 区分：risk-averse 更强调不愿冒险。
+同义替换/错误选项信号：cautious; conservative; unwilling to take risks
+多场景例句：risk-averse investors；a risk-averse culture；risk-averse decision-making
+其他可用地方：职场发展、创业、经济政策</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -212,17 +295,28 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>commercialise research</t>
+          <t>complement one another</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：将科研成果商业化。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：把知识、实验室成果或发明转化为产品、企业和市场价值。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：中性偏积极，但也可能引出学术与商业的张力。</t>
+          <t>字面含义：相互补充
+考研核心考点：议论文关系表达
+词汇拆解：complement = 补充；one another = 彼此
+熟词辟义/一词多义：complement 不是 compliment（称赞）。
+语气色彩：正式、正面</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Boston commercialises it better. 波士顿不一定科研更密集，但更会把科研变成产业。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：知识本身不等于社会影响，转化能力也关键。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Universities should commercialise research without sacrificing academic independence.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：A discovery changes society only when it can be commercialised responsibly.&lt;br&gt;&lt;b&gt;例句3 经济&lt;/b&gt;：Countries that fail to commercialise research may lose the value of their own inventions.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技创新、大学功能、经济发展、社会责任。</t>
+          <t>文章语境：文章说两个 Cambridge 的优势和弱点可以相互补足。
+暗示意思/政治意味/诙谐意味：暗示竞争之外还有合作与互补。
+特殊考查方式：阅读结构题可判断不是简单对立，而是互补关系。
+答题技巧：注意拼写：complement 补充，compliment 赞美。
+同义替换/错误选项信号：supplement each other; work together; be mutually reinforcing
+多场景例句：universities and firms complement one another；capital and talent complement one another；tradition and innovation can complement each other
+其他可用地方：文化交流、教育合作、职场协作
+归一化合并：本卡覆盖这些变体：complement one another</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -234,17 +328,28 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>be constrained by</t>
+          <t>lure talent across the pond</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：受制于，被……限制。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式，常用于结构性限制，不只是个人困难。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：constrained by resources / infrastructure / rules / time / tradition。</t>
+          <t>字面含义：吸引人才跨越大西洋
+考研核心考点：lure + 宾语 + 方向，外刊常用
+词汇拆解：lure = attract/tempt；talent = 人才；across the pond = 跨越大西洋
+熟词辟义/一词多义：lure 可带诱惑色彩，不只是普通 attract。
+语气色彩：新闻语体，中性略带策略意味</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Cambridge remains constrained by its medieval skin. 作者用 medieval skin 形象说明老城空间限制创新扩张。&lt;br&gt;&lt;b&gt;暗示/诙谐&lt;/b&gt;：历史底蕴既是魅力，也是束缚。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Many students are constrained by limited access to quality resources.&lt;br&gt;&lt;b&gt;例句2 城市&lt;/b&gt;：Historic cities are often constrained by old infrastructure.&lt;br&gt;&lt;b&gt;例句3 个人&lt;/b&gt;：A person should not be constrained by past failures.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育公平、城市发展、个人成长、经济转型。</t>
+          <t>文章语境：文章讨论英美 Cambridge 互相吸引人才流动。
+暗示意思/政治意味/诙谐意味：暗示人才竞争是创新地理变化的核心。
+特殊考查方式：细节题可能用 attract/recruit 替换 lure。
+答题技巧：lure 后直接接人或资源；不要译成“诱饵人才”。
+同义替换/错误选项信号：attract talent; draw talent; recruit talent; tempt talent away
+多场景例句：lure talent across the pond；lure scientists from rival hubs；lure young graduates into biotech
+其他可用地方：教育、职场发展、国际交流
+归一化合并：本卡覆盖这些变体：lure talent；lure across talent；across the pond</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -256,17 +361,27 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>medieval skin</t>
+          <t>plaque</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：中世纪外壳。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：历史城市的旧空间、旧街区、旧基础设施。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：形象、略带诙谐：把城市比作有一层老皮肤。</t>
+          <t>字面含义：纪念牌；匾牌；牙菌斑
+考研核心考点：熟词僻义与多义
+词汇拆解：plaque = flat sign/tablet；medical plaque = 斑块/牙菌斑
+熟词辟义/一词多义：外刊城市语境多为“纪念牌”，医学语境可为“斑块”。
+语气色彩：中性，文化/医学语境不同</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：the real Cambridge remains constrained by its medieval skin. 剑桥的历史风貌限制住房、水、交通和实验室空间。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：传统不是纯粹加分项，也可能限制现代创新。&lt;br&gt;&lt;b&gt;例句1 文化&lt;/b&gt;：A city should protect its historical skin without letting it block modern life.&lt;br&gt;&lt;b&gt;例句2 科技&lt;/b&gt;：Innovation cannot thrive if it is trapped in a medieval skin of outdated infrastructure.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：Tradition should be preserved, but not allowed to become a skin that prevents renewal.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：传统文化创新、城市发展、环境规划、科技基础设施。</t>
+          <t>文章语境：文章用 plaque 指城市中标记创新历史的纪念牌。
+暗示意思/政治意味/诙谐意味：暗示城市把科学成就包装成可参观的创新叙事。
+特殊考查方式：词义题看语境：city/history 通常是纪念牌；health 是斑块。
+答题技巧：不要一看到 plaque 就译“牙菌斑”。
+同义替换/错误选项信号：commemorative plaque; marker; tablet; memorial sign
+多场景例句：a plaque marking a discovery；a blue plaque on a building；arterial plaque in a health article
+其他可用地方：文化、历史、健康医学</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -278,17 +393,28 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>be starved of</t>
+          <t>in-vitro fertilisation</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：严重缺乏，得不到足够供应。&lt;br&gt;&lt;b&gt;本义&lt;/b&gt;：starve = 挨饿。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：资金、空间、人才、关注、资源等被“饿着”。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：比 lack 强烈，形象。</t>
+          <t>字面含义：体外受精；试管婴儿技术
+考研核心考点：医学科技主题词
+词汇拆解：in vitro = 在玻璃中/体外；fertilisation = 受精
+熟词辟义/一词多义：vitro 常见于医学实验语境，不是普通生活词。
+语气色彩：正式、医学科技语体</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Britain's Cambridge is starved of capital and space. 英国剑桥不是一般缺，而是发展被资源饥饿限制。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：科研强但成长营养不足。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Rural schools are often starved of qualified teachers.&lt;br&gt;&lt;b&gt;例句2 创业&lt;/b&gt;：Promising startups may fail if they are starved of long-term capital.&lt;br&gt;&lt;b&gt;例句3 个人&lt;/b&gt;：Young people starved of encouragement may lose confidence.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育资源、经济发展、心理成长、科技创新。</t>
+          <t>文章语境：文章提到剑桥创新历史中与 IVF 相关的成果。
+暗示意思/政治意味/诙谐意味：暗示大学城创新可带来改变社会和家庭生活的医学突破。
+特殊考查方式：细节题可能用 IVF 缩写替换。
+答题技巧：记住 in-vitro fertilisation = IVF，不要拆开死译。
+同义替换/错误选项信号：IVF; assisted reproduction; fertility treatment
+多场景例句：in-vitro fertilisation research；a breakthrough in IVF；commercialise fertility technology
+其他可用地方：健康、科技生活、医学伦理
+归一化合并：本卡覆盖这些变体：vitro fertilisation</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -300,17 +426,27 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>a dearth of</t>
+          <t>a global hub for</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：缺乏，匮乏。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式书面，常接抽象资源。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：a dearth of capital / evidence / talent / trust / imagination。</t>
+          <t>字面含义：全球……中心
+考研核心考点：城市/产业定位高频表达
+词汇拆解：global = 全球的；hub = 枢纽/中心；for 后接领域
+熟词辟义/一词多义：hub 原指轮毂/枢纽，引申为活动中心。
+语气色彩：正式、正面</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：a dearth of domestic capital later on means firms fall behind as they grow. 后期本土资本不足导致企业成长受限。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：早期热闹不代表能长大，长期支持更重要。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：A dearth of reading habits can weaken students' language ability.&lt;br&gt;&lt;b&gt;例句2 社会&lt;/b&gt;：A dearth of trust makes public cooperation difficult.&lt;br&gt;&lt;b&gt;例句3 科技&lt;/b&gt;：A dearth of patient capital can slow the commercialisation of research.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育学习、社会信任、科技创新、经济发展。</t>
+          <t>文章语境：文章称 Cambridge 是全球创新或生物科技中心。
+暗示意思/政治意味/诙谐意味：暗示资源、人才、资本在此集中。
+特殊考查方式：写作可替换 important centre。
+答题技巧：hub 后常接 for/of：a hub for innovation。
+同义替换/错误选项信号：global centre; international hub; leading centre
+多场景例句：a global hub for biotech；a hub for innovation and talent；a global centre of academic excellence
+其他可用地方：城市发展、科技、教育</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -322,17 +458,27 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>proof of concept</t>
+          <t>namesake</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：概念验证，初步证明想法可行。&lt;br&gt;&lt;b&gt;技术/创业语境&lt;/b&gt;：不是最终产品，而是证明方向能跑通。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：商业、技术、科研高频。</t>
+          <t>字面含义：同名者；同名地
+考研核心考点：文化比较和历史渊源词
+词汇拆解：name + sake；同名的人/地/机构
+熟词辟义/一词多义：namesake 不等于 nickname，是“同名对象”。
+语气色彩：书面、文化类常用</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：疫情期间美国一些公司 often without proof of concept 就过早 IPO。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：资本过热会让尚未验证的想法过早进入市场。&lt;br&gt;&lt;b&gt;例句1 科技&lt;/b&gt;：A new technology should not be scaled up without proof of concept.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：Pilot programmes can provide proof of concept before reform is expanded nationwide.&lt;br&gt;&lt;b&gt;例句3 职场&lt;/b&gt;：A small project can serve as proof of concept for a larger plan.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技创新、教育改革、创业、项目管理。</t>
+          <t>文章语境：文章用 American namesake 指美国马萨诸塞州剑桥。
+暗示意思/政治意味/诙谐意味：暗示同名背后有历史移植、大学传统和文化连接。
+特殊考查方式：细节题会考 namesake 指代哪个 Cambridge。
+答题技巧：遇到 namesake 先回看前文名字。
+同义替换/错误选项信号：same-named counterpart; counterpart with the same name
+多场景例句：its American namesake；a city and its namesake across the Atlantic；borrow prestige from a famous namesake
+其他可用地方：文化交流、历史、城市比较</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -344,17 +490,27 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>risk-averse</t>
+          <t>involved in founding Harvard College</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：规避风险的，风险厌恶的。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济金融常用，不一定贬义；但过度 risk-averse 会抑制创新。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：risk-averse investors / parents / institutions / students。</t>
+          <t>字面含义：参与创办哈佛学院的
+考研核心考点：过去分词后置定语
+词汇拆解：involved in = 参与；founding = 创办；Harvard College = 哈佛学院
+熟词辟义/一词多义：found 作动词是“创立”，不是 find 的过去式 found。
+语气色彩：正式、历史叙述</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Investors became more risk-averse, giving larger amounts to fewer firms. 投资人更谨慎，把钱集中给少数公司。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：市场低迷后，资本不是消失，而是更挑剔。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Overly risk-averse students may avoid challenges that help them grow.&lt;br&gt;&lt;b&gt;例句2 投资&lt;/b&gt;：Risk-averse investors prefer proven business models.&lt;br&gt;&lt;b&gt;例句3 作文&lt;/b&gt;：A society that is too risk-averse may fail to encourage creativity.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：个人品质、创新精神、职场发展、经济生活。</t>
+          <t>文章语境：文章说 many involved in founding Harvard College were Cambridge alumni。
+暗示意思/政治意味/诙谐意味：暗示美国剑桥与英国剑桥的教育渊源。
+特殊考查方式：长难句考分词后置定语：Many involved in... = Many who were involved in...
+答题技巧：看到 involved in doing 作后置定语，先还原成 who were involved in doing。
+同义替换/错误选项信号：who took part in founding; those connected with founding
+多场景例句：people involved in founding a college；scholars involved in building an institution；alumni involved in educational reform
+其他可用地方：教育、文化交流、长难句</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -366,17 +522,28 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>complement one another</t>
+          <t>alumni, not aluminium</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：相互补充。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：两个事物不是替代关系，而是各自弥补对方短板。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：积极、理性，适合写平衡观点。</t>
+          <t>字面含义：alumni = 校友，不是 aluminum/aluminium 铝
+考研核心考点：形近词辨析
+词汇拆解：alumnus 单数男校友；alumna 女校友；alumni 复数/泛指校友；aluminium/aluminum = 铝
+熟词辟义/一词多义：alumni 与 aluminum/aluminium 拼写接近但意思完全不同。
+语气色彩：正式、教育语境</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：two Cambridges' strengths and weaknesses seem to complement one another. 英国科研强、美国商业化强，正好互补。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：合作来自结构互补，不是单纯友好。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Online learning and traditional classrooms can complement one another.&lt;br&gt;&lt;b&gt;例句2 职场&lt;/b&gt;：Technical skills and communication skills complement one another.&lt;br&gt;&lt;b&gt;例句3 文化&lt;/b&gt;：Tradition and innovation can complement one another if handled wisely.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育、职场、文化交流、科技发展。</t>
+          <t>文章语境：文章说 Cambridge alumni 参与创办 Harvard。
+暗示意思/政治意味/诙谐意味：暗示大学的人才网络会跨地区复制制度。
+特殊考查方式：词义题/翻译题易误读形近词。
+答题技巧：看到 alumni 立即译“校友”，不要联想到金属铝。
+同义替换/错误选项信号：graduates; former students; university alumni
+多场景例句：Cambridge alumni；an alumni network；alumni involved in founding a college
+其他可用地方：教育、人脉、文化传承
+归一化合并：本卡覆盖这些变体：aluminum/alumni</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -388,17 +555,27 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>lure talent</t>
+          <t>imitate</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：吸引人才。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：lure 本义有“诱饵、引诱”，比 attract 更有策略性和竞争意味。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：新闻英语，常用于城市、公司、国家争夺人才。</t>
+          <t>字面含义：模仿；仿效
+考研核心考点：比较文章中的行为动词
+词汇拆解：imitate = copy/follow as a model
+熟词辟义/一词多义：可中性，也可暗示缺乏原创。
+语气色彩：中性到略贬，取决于上下文</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：美国削减公共研究经费 may help Britain lure across talent. 英国可能趁机吸引人才跨洋而来。&lt;br&gt;&lt;b&gt;政治意味&lt;/b&gt;：人才流动受国家政策影响，是国际竞争的一部分。&lt;br&gt;&lt;b&gt;例句1 职场&lt;/b&gt;：Companies lure talent with flexible work and meaningful projects.&lt;br&gt;&lt;b&gt;例句2 教育&lt;/b&gt;：World-class universities can lure talent from around the globe.&lt;br&gt;&lt;b&gt;例句3 国家竞争&lt;/b&gt;：Stable research funding helps a country lure and retain scientific talent.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：职场发展、教育强国、科技竞争、城市吸引力。</t>
+          <t>文章语境：文章讨论美国剑桥并非只是模仿英国剑桥。
+暗示意思/政治意味/诙谐意味：暗示继承者可能超越原型。
+特殊考查方式：主旨题会考 imitate 与 surpass 的对比。
+答题技巧：注意 imitate 不等于 innovate；两者常形成对比。
+同义替换/错误选项信号：copy; emulate; model itself on; follow the example of
+多场景例句：imitate a successful model；not merely imitate the West；imitate without understanding the context
+其他可用地方：文化交流、教育改革、创新</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -410,17 +587,27 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>The former..., the latter...</t>
+          <t>mush into</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：前者……，后者……。&lt;br&gt;&lt;b&gt;语法&lt;/b&gt;：former 指前面两个对象中的第一个；latter 指第二个。&lt;br&gt;&lt;b&gt;功能&lt;/b&gt;：避免重复名词，让比较更紧凑。</t>
+          <t>字面含义：糊成一团；混成难分的整体
+考研核心考点：形象动词短语
+词汇拆解：mush = 糊状物；mush into = blend messily into
+熟词辟义/一词多义：mush 带不清晰、边界模糊的感觉。
+语气色彩：口语化、形象、略调侃</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：The former offers access to America's capital and market; the latter, world-class talent on the cheap. 前者指美国办公室，后者指英国本土研发。&lt;br&gt;&lt;b&gt;例句1 教育&lt;/b&gt;：Online courses offer flexibility; traditional classrooms offer discipline. The former saves time; the latter builds routine.&lt;br&gt;&lt;b&gt;例句2 职场&lt;/b&gt;：Hard skills and soft skills are both necessary. The former helps one do the job; the latter helps one work with people.&lt;br&gt;&lt;b&gt;例句3 写作&lt;/b&gt;：Economic growth and environmental protection should not be opposed. The former creates resources; the latter protects the future.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：所有对比类作文。</t>
+          <t>文章语境：文章用它描述两个 Cambridge 的故事或身份可能混在一起。
+暗示意思/政治意味/诙谐意味：暗示相似性强到容易混淆。
+特殊考查方式：词义题考形象引申义。
+答题技巧：不要译成“蘑菇进”，应译“混成/糊成”。
+同义替换/错误选项信号：merge into; blur into; blend into
+多场景例句：mush into one narrative；two identities mush into each other；facts and myths mush into a single story
+其他可用地方：文化比较、媒体叙事、写作修辞</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -432,17 +619,27 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>The two Cambridges: central argument</t>
+          <t>a curated "innovation trail"</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;中心论点&lt;/b&gt;：顶级创新生态不只靠大学和科研，还需要资本、基础设施、市场、临床试验能力和跨区域合作。英国剑桥科研强但资源受限，美国剑桥商业化强但受资本泡沫影响，二者正在互补。</t>
+          <t>字面含义：精心策划的“创新路线/创新步道”
+考研核心考点：curated 的熟词新义
+词汇拆解：curate 本义策展；curated = 精选并组织好的
+熟词辟义/一词多义：curated 不只是博物馆策展，也可指人为筛选包装的信息/路线。
+语气色彩：文化营销语体，略带包装感</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>&lt;b&gt;可背作文论点&lt;/b&gt;：Innovation depends not only on talent, but also on institutions, infrastructure and long-term support.&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A successful city turns knowledge into social value by connecting education, capital and public services.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Research can change the world only when ideas are supported by patient capital and practical infrastructure.&lt;br&gt;&lt;b&gt;例句3&lt;/b&gt;：Cooperation works best when different sides complement, rather than duplicate, one another.&lt;br&gt;&lt;b&gt;适用话题&lt;/b&gt;：教育学习、科技创新、经济发展、职场生活、文化交流。</t>
+          <t>文章语境：文章提到剑桥用创新路线展示科学成就。
+暗示意思/政治意味/诙谐意味：暗示城市将创新历史转化为品牌叙事。
+特殊考查方式：词义题可能考 curated = carefully selected/organised。
+答题技巧：不要译为“治疗过的”，译为“策划/精选的”。
+同义替换/错误选项信号：carefully selected; organised; packaged; branded
+多场景例句：a curated innovation trail；a curated list of start-ups；a curated cultural route
+其他可用地方：文化、城市品牌、科技传播</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -454,17 +651,28 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>shape sb/sth</t>
+          <t>dub A B</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：塑造，影响……的形成。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：shape 不只是“形状”，作动词表示长期塑造。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：教育、文化、历史、人格话题高频。</t>
+          <t>字面含义：把 A 称为 B；给 A 起名为 B
+考研核心考点：新闻报道高频动词
+词汇拆解：dub + object + name/title
+熟词辟义/一词多义：dub 不只是“配音”，新闻中常指“称作/封为”。
+语气色彩：新闻语体、中性</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Its university shaped Milton, Darwin and Hawking。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Education shapes not only knowledge but also character.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Family, school and society shape a young person's values.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育学习、精神品质、文化影响。</t>
+          <t>文章语境：文章可能用 dubbed 引出某个称号或路线名称。
+暗示意思/政治意味/诙谐意味：暗示媒体或机构在塑造标签。
+特殊考查方式：语法题考双宾/宾补结构。
+答题技巧：看到 dub A B，译成“把 A 称为 B”。
+同义替换/错误选项信号：call A B; label A B; name A B
+多场景例句：dub the area an innovation cluster；be dubbed a global hub；dub the route an innovation trail
+其他可用地方：媒体表达、文化传播、城市品牌
+归一化合并：本卡覆盖这些变体：dub</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -476,17 +684,27 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>mark where</t>
+          <t>almost identical</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：标明……发生的地点。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：历史叙述常用。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：a plaque marks where...</t>
+          <t>字面含义：几乎完全相同
+考研核心考点：比较类形容词短语
+词汇拆解：almost = 几乎；identical = 完全相同的
+熟词辟义/一词多义：identical 比 similar 更强，表示高度一致。
+语气色彩：中性、强调相似度高</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：A plaque outside the Eagle pub marks where DNA discovery was announced。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A museum can mark where important cultural exchanges began.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Public memorials mark where society learned painful lessons.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：文化、历史、城市介绍。</t>
+          <t>文章语境：文章比较两个 Cambridge 的名字、大学气质或创新叙事相似。
+暗示意思/政治意味/诙谐意味：暗示表面相似可能掩盖深层差异。
+特殊考查方式：细节题可能用 nearly the same 替换。
+答题技巧：identical 不要弱译成“一点像”。
+同义替换/错误选项信号：nearly the same; virtually identical; almost the same
+多场景例句：almost identical names；almost identical strategies；almost identical problems beneath different surfaces
+其他可用地方：比较写作、文化交流、科技政策</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -498,17 +716,27 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>birthplace of</t>
+          <t>exploit each other's weaknesses</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：……的诞生地。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：某项技术、思想、运动或制度最早出现的地方。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：文化/科技介绍高频。</t>
+          <t>字面含义：利用彼此的弱点
+考研核心考点：exploit 的熟词僻义
+词汇拆解：exploit = 利用/开发；weaknesses = 弱点
+熟词辟义/一词多义：exploit 可中性“利用资源”，也可负面“剥削/钻空子”。
+语气色彩：策略性、略负面</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Cambridge is the birthplace of IVF and key biotech designs。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Universities can become the birthplace of new ideas.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：The city is often described as the birthplace of modern industry.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技创新、文化交流、城市写作。</t>
+          <t>文章语境：文章说两地可利用对方短板形成机会。
+暗示意思/政治意味/诙谐意味：暗示竞争关系中弱点也会变成对方的机会。
+特殊考查方式：态度题需判断 exploit 褒贬。
+答题技巧：科技/商业语境常译“利用”，社会伦理语境可译“剥削”。
+同义替换/错误选项信号：take advantage of; make use of; capitalise on
+多场景例句：exploit each other's weaknesses；exploit a rival's shortage of capital；exploit gaps in regulation
+其他可用地方：商业竞争、职场策略、公共伦理</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -520,17 +748,27 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>global hub for</t>
+          <t>increasingly conjoined</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：……的全球中心。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济/城市/科技报道常用。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：a global hub for finance / culture / AI / life sciences。</t>
+          <t>字面含义：日益连接在一起；越来越紧密相连
+考研核心考点：趋势表达 + 正式形容词
+词汇拆解：increasingly = 越来越；conjoined = joined together
+熟词辟义/一词多义：conjoined 可指身体连体，也可抽象指系统/命运相连。
+语气色彩：正式、形象</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Cambridge is a global hub for life sciences, semiconductors and AI。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A city can become a global hub for innovation by attracting talent.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Universities help turn local communities into global hubs for research.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：城市发展、科技、教育、经济。</t>
+          <t>文章语境：文章说两个创新生态越来越互相连接。
+暗示意思/政治意味/诙谐意味：暗示未来不是各自独立，而是跨大西洋共同运作。
+特殊考查方式：主旨题可替换为 more closely connected。
+答题技巧：译出趋势：日益/越来越。
+同义替换/错误选项信号：more closely linked; increasingly connected; tied together
+多场景例句：increasingly conjoined innovation systems；economies increasingly conjoined by trade；education and technology increasingly connected
+其他可用地方：全球化、科技合作、文化交流</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
@@ -542,17 +780,27 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>echoed by</t>
+          <t>bump into one another</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：被……呼应，被……映照。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：echo 不只是回声，也可指相似现象在另一处出现。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：文雅，适合写文化联系。</t>
+          <t>字面含义：偶然碰见彼此；意外交汇
+考研核心考点：短语动词，表示偶遇或互动增加
+词汇拆解：bump = 撞；bump into = 偶然遇见
+熟词辟义/一词多义：不只指身体碰撞，也指人、机构、生态发生交集。
+语气色彩：口语化、形象</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Cambridge's successes are echoed by its American namesake。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A city's educational success may be echoed by its industries.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Traditional values are echoed in modern volunteer work.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：文化交流、教育影响、历史延续。</t>
+          <t>文章语境：文章用它描述两地人才、资本、公司越来越常相遇。
+暗示意思/政治意味/诙谐意味：暗示创新网络密度提高，偶遇本身也创造机会。
+特殊考查方式：词义题可能考 bump into = encounter by chance。
+答题技巧：不要死译“撞进彼此”。
+同义替换/错误选项信号：run into; encounter; cross paths with
+多场景例句：bump into one another at conferences；start-ups and investors bump into one another；ideas bump into one another in a dense cluster
+其他可用地方：职场社交、创新生态、文化交流</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
@@ -564,17 +812,27 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>alma mater</t>
+          <t>unicorns (private firms worth more than $1bn)</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：母校。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式/文雅，有情感和身份归属意味。&lt;br&gt;&lt;b&gt;常见&lt;/b&gt;：return to one's alma mater。</t>
+          <t>字面含义：独角兽企业：估值超过 10 亿美元的未上市公司
+考研核心考点：商业科技报道核心词
+词汇拆解：unicorn = 神话独角兽；商业中指 rare high-value private firm
+熟词辟义/一词多义：不是动物，而是高估值未上市公司。
+语气色彩：创业/投资语体</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：colonists renamed the settlement to honour their alma mater。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Graduates often feel a lifelong bond with their alma mater.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A strong alma mater can connect people across countries and generations.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育、文化传承、身份认同。</t>
+          <t>文章语境：文章用 unicorns 衡量创新生态中高成长企业数量。
+暗示意思/政治意味/诙谐意味：暗示资本市场和创业生态的成熟度。
+特殊考查方式：细节题可能考括号解释。
+答题技巧：看到括号定义要直接吸收为考点。
+同义替换/错误选项信号：billion-dollar start-up; high-value private firm; private firm worth over $1bn
+多场景例句：produce more unicorns；a cluster full of unicorns；turn research into unicorn companies
+其他可用地方：经济、创业、科技创新</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -586,17 +844,27 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>curated trail</t>
+          <t>venture-capital (VC) deals</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：精心设计/策划的路线。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：curate 原指策展，引申为筛选、组织、策划内容。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：文化、旅游、知识管理常用。</t>
+          <t>字面含义：风险投资交易
+考研核心考点：创业金融核心搭配
+词汇拆解：venture = 风险企业；capital = 资本；deal = 交易/投资项目
+熟词辟义/一词多义：deal 不只是“交易”，投资语境指一笔融资。
+语气色彩：正式商业语体</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：a curated innovation trail 展示波士顿-剑桥创新历史。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A curated reading list can help students learn more efficiently.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Museums use curated routes to tell a coherent story.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：学习规划、文化旅游、知识管理。</t>
+          <t>文章语境：文章比较两地获得 VC deals 的数量和规模。
+暗示意思/政治意味/诙谐意味：暗示资本供给决定科研能否变成公司。
+特殊考查方式：细节题会用 investment rounds/funding deals 替换。
+答题技巧：VC = venture capital；不要译为“冒险资本交易”。
+同义替换/错误选项信号：VC investment; funding round; start-up financing
+多场景例句：venture-capital deals in biotech；attract more VC deals；larger VC deals for fewer firms
+其他可用地方：经济、创业、科技商业化</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -608,17 +876,27 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>dubbed</t>
+          <t>be home to</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：被称为，被冠以……称号。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：新闻高频，常用于外号、称号、媒体标签。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：be dubbed the world's most...</t>
+          <t>字面含义：是……所在地；拥有/孕育
+考研核心考点：地点介绍高频表达
+词汇拆解：home 不只是家，可指所在地/大本营。
+熟词辟义/一词多义：be home to + 机构/群体/产业
+语气色彩：正式、中性正面</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Kendall Square is dubbed the world's most innovative square mile。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：The city has been dubbed a global centre of technology.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Some students are dubbed digital natives, but they still need guidance.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：新闻阅读、城市介绍、科技文化。</t>
+          <t>文章语境：文章介绍 Cambridge is home to universities, firms or labs。
+暗示意思/政治意味/诙谐意味：暗示地方承载某种资源或身份。
+特殊考查方式：写作替换 there are。
+答题技巧：不要译成“是……的家”太生硬，译“坐落着/拥有”。
+同义替换/错误选项信号：host; contain; be the site of; house
+多场景例句：be home to world-class universities；be home to biotech start-ups；a city home to pools of talent
+其他可用地方：城市介绍、教育、科技产业</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
@@ -630,17 +908,28 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>primarily driven by</t>
+          <t>build on these advantages</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：主要由……驱动。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式分析句型。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：be driven by demand / talent / technology / research。</t>
+          <t>字面含义：建立在这些优势之上；利用这些优势继续发展
+考研核心考点：发展逻辑表达
+词汇拆解：build on = use as a foundation；advantages = 优势
+熟词辟义/一词多义：build on 不是“在上面建房”，而是“基于……推进”。
+语气色彩：正式、中性</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：innovation engines driven primarily by academic research。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Economic growth should be driven by innovation rather than speculation.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Learning is driven primarily by curiosity and discipline.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济、教育、科技、个人成长。</t>
+          <t>文章语境：文章说明美国剑桥在已有大学、资本、人才优势上继续扩张。
+暗示意思/政治意味/诙谐意味：暗示成功是累积过程，不是单点突破。
+特殊考查方式：写作可用于承接前文优势。
+答题技巧：注意介词 on，不是 build advantages。
+同义替换/错误选项信号：capitalize on; make use of; develop from; rest on
+多场景例句：build on these advantages；build on academic strength；build on existing talent pools
+其他可用地方：教育、职场成长、科技创新
+归一化合并：本卡覆盖这些变体：built on these advantages</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -652,17 +941,27 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>per person</t>
+          <t>an infusion of capital</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：按人均计算。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：用于把不同规模地区放在同一标准下比较。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：数据阅读高频。</t>
+          <t>字面含义：资本注入
+考研核心考点：经济金融类高频名词短语
+词汇拆解：infusion = 注入；capital = 资本
+熟词辟义/一词多义：infusion 可指液体注入，也可指资金/能量注入。
+语气色彩：正式、经济语体</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：alumni founders per person, innovation clusters per person。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Income per person is not the same as quality of life.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Reading hours per person can reflect a society's learning culture.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：图表作文、经济数据、阅读理解。</t>
+          <t>文章语境：文章说资本注入帮助美国剑桥企业成长。
+暗示意思/政治意味/诙谐意味：暗示钱不是唯一因素，但能放大科研优势。
+特殊考查方式：细节题会用 injection of funding 替换。
+答题技巧：infusion of 后接 capital/funds/energy。
+同义替换/错误选项信号：injection of capital; influx of funding; fresh investment
+多场景例句：an infusion of capital；a fresh infusion of funding；capital infusion into start-ups
+其他可用地方：经济、创业、公共投资</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
@@ -674,17 +973,27 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>depends on what you count</t>
+          <t>headquarters</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：取决于你计算什么。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：排名或结论受指标影响。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：批判数据口径，外刊常用思路。</t>
+          <t>字面含义：总部；总公司所在地
+考研核心考点：商业组织词
+词汇拆解：head + quarters；常作单复同形名词
+熟词辟义/一词多义：headquarters 形式像复数，但可指一个总部。
+语气色彩：正式、中性</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：which Cambridge comes first depends on what you count。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Whether online learning is better depends on what you count: scores, flexibility or motivation.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A city's success depends on what you count, GDP or well-being.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：图表分析、教育评价、社会发展。</t>
+          <t>文章语境：文章提到公司总部是否留在 Cambridge。
+暗示意思/政治意味/诙谐意味：暗示企业从实验室成长为成熟公司的地点选择。
+特殊考查方式：细节题可问 companies base their headquarters where。
+答题技巧：注意 headquarters 常与 locate/base/move 搭配。
+同义替换/错误选项信号：corporate base; head office; main office
+多场景例句：company headquarters；move headquarters to Boston；keep headquarters near the university
+其他可用地方：职场、商业、城市经济</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
@@ -696,17 +1005,27 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>patent awards</t>
+          <t>Cows still graze in the city centre</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：专利授权。&lt;br&gt;&lt;b&gt;注意&lt;/b&gt;：award 这里不是奖品，而是授予/批准。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：科技创新和知识产权常用。</t>
+          <t>字面含义：奶牛仍在市中心吃草
+考研核心考点：具体画面表达 + 对比修辞
+词汇拆解：graze = 吃草；city centre = 市中心
+熟词辟义/一词多义：graze 不只是擦伤，也可指牲畜吃草。
+语气色彩：形象、略幽默</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Global Innovation Index counts patent awards。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Patent awards can reflect a country's research output.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Innovation should be measured not only by patent awards but also by social impact.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技创新、知识产权、经济发展。</t>
+          <t>文章语境：文章用这句话突出英国剑桥古老、乡村化空间与高科技野心并存。
+暗示意思/政治意味/诙谐意味：暗示传统城市肌理会限制现代产业扩张。
+特殊考查方式：推理题考这类细节服务于什么论点。
+答题技巧：不要只当风景描写，它在论证“空间受限/城市保守”。
+同义替换/错误选项信号：cows grazing downtown; pastoral scenes in an urban centre
+多场景例句：cows still graze in the city centre；old streets constrain modern labs；pastoral charm limits industrial scale
+其他可用地方：城市发展、传统与现代、环境</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
@@ -718,17 +1037,27 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>venture-capital deals</t>
+          <t>a shortage of facilities</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：风险投资交易。&lt;br&gt;&lt;b&gt;组成&lt;/b&gt;：venture capital = 风投；deal = 交易/融资事件。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：商业外刊高频。</t>
+          <t>字面含义：设施短缺
+考研核心考点：资源不足类表达
+词汇拆解：shortage = 短缺；facilities = 设施/场地/设备
+熟词辟义/一词多义：facilities 不只是“便利”，常指教学、科研、生产设施。
+语气色彩：正式、负面</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：WIPO 用 VC deals 衡量创新密度。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Venture-capital deals can help startups turn research into products.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Too many venture-capital deals may also create bubbles.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济、科技创业、商业化。</t>
+          <t>文章语境：文章说科研企业缺少实验室等设施。
+暗示意思/政治意味/诙谐意味：暗示创新生态不只需要人才，还需要物理空间。
+特殊考查方式：原因题定位 shortage of 后面的名词。
+答题技巧：shortage of + 资源 是作文高频结构。
+同义替换/错误选项信号：lack of facilities; insufficient facilities; scarcity of lab space
+多场景例句：a shortage of facilities；a shortage of lab space；schools facing a shortage of sports facilities
+其他可用地方：教育资源、科技产业、城市规划</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
@@ -740,17 +1069,27 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>reverse the order</t>
+          <t>makeshift labs</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：颠倒顺序。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：换一个评价指标，排名结果完全不同。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：数据对比常用。</t>
+          <t>字面含义：临时搭建的实验室；简易实验室
+考研核心考点：形容资源不足的具体搭配
+词汇拆解：makeshift = 临时凑合的；labs = laboratories
+熟词辟义/一词多义：makeshift 带“将就、非正式、条件不足”的意味。
+语气色彩：负面、形象</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Dealroom reverses the order: Boston-Cambridge wins by enterprise value and unicorns。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A different standard may reverse the order of the ranking.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：If we value health more than speed, modern life may reverse the order of priorities.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：图表作文、比较论证、价值排序。</t>
+          <t>文章语境：文章用 makeshift labs 描述英国剑桥空间和设施不足。
+暗示意思/政治意味/诙谐意味：暗示高水平科研被迫在低配空间中运转。
+特殊考查方式：态度题显示作者认为条件不理想。
+答题技巧：译出“临时/简易/凑合”，不要只译“实验室”。
+同义替换/错误选项信号：temporary labs; improvised laboratories; ad hoc facilities
+多场景例句：makeshift labs in old buildings；makeshift classrooms；improvised workspaces for start-ups
+其他可用地方：教育设施、科研条件、创业</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
@@ -762,17 +1101,28 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>relative to</t>
+          <t>hemmed in by</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：相对于，与……相比。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式，数据比较高频。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：relative to population / income / size / cost。</t>
+          <t>字面含义：被……包围/限制住
+考研核心考点：空间限制和制度限制都可用
+词汇拆解：hem = 包边；hem in = 围住、限制
+熟词辟义/一词多义：可指地理上被围住，也可指选择被限制。
+语气色彩：形象、负面</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：more patents relative to population size。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A student's progress should be judged relative to his starting point.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：The cost of education is high relative to family income.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：图表、教育评价、经济阅读。</t>
+          <t>文章语境：文章说 Cambridge hemmed in by old city fabric/space constraints。
+暗示意思/政治意味/诙谐意味：暗示城市魅力同时成为发展束缚。
+特殊考查方式：词义题可能考 from physical enclosure to constraint。
+答题技巧：by 后面是限制来源。
+同义替换/错误选项信号：be boxed in by; be constrained by; be surrounded by
+多场景例句：hemmed in by old streets；hemmed in by regulations；a start-up hemmed in by high rents
+其他可用地方：城市发展、政策限制、职场困境
+归一化合并：本卡覆盖这些变体：Hemmed</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
@@ -784,17 +1134,27 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>scale</t>
+          <t>Google's venture arm</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：规模。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：不是天平/刻度，而是经济或组织规模。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：规模带来的市场、人才、资本和基础设施优势。</t>
+          <t>字面含义：谷歌的风险投资部门
+考研核心考点：商业组织结构词
+词汇拆解：venture arm = corporate investment unit；arm = 部门/分支
+熟词辟义/一词多义：arm 不只是胳膊，也指机构分支。
+语气色彩：正式商业语体</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：American Cambridge is more advanced mostly because of scale。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Scale can turn a good idea into a powerful industry.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Small schools lack scale, but they may offer closer relationships.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济发展、教育机构、企业成长。</t>
+          <t>文章语境：文章引用 Google's venture arm 的人评价剑桥生态。
+暗示意思/政治意味/诙谐意味：暗示大科技公司通过投资部门参与创新生态。
+特殊考查方式：词义题考 arm 的机构义。
+答题技巧：看到 company + arm，译为“……部门/分支”。
+同义替换/错误选项信号：investment arm; venture unit; corporate VC division
+多场景例句：Google's venture arm；a bank's research arm；a university's commercialisation arm
+其他可用地方：商业、科技投资、组织结构</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
@@ -806,17 +1166,28 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>build on advantages</t>
+          <t>put it differently</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：在优势基础上继续发展。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：积极，发展策略常用。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：build on strengths / success / existing advantages。</t>
+          <t>字面含义：换句话说；换个说法
+考研核心考点：解释重述标记
+词汇拆解：put = express；put it differently = express it in another way
+熟词辟义/一词多义：put 不只是放置，可表示“表达”。
+语气色彩：口语化但外刊常用</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Massachusetts has built on these advantages。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Students should build on their strengths while fixing weaknesses.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Cities can build on educational advantages to attract industry.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：学习规划、城市发展、职场成长。</t>
+          <t>文章语境：文章用它引出对问题的另一种概括。
+暗示意思/政治意味/诙谐意味：暗示后文是作者或受访者的重新表述。
+特殊考查方式：结构题可判断同义解释。
+答题技巧：看到 put it differently，后面通常不是新论点，而是重述。
+同义替换/错误选项信号：in other words; to put it another way; differently stated
+多场景例句：put it differently；to put the problem differently；put the contrast in simpler terms
+其他可用地方：写作连接、阅读结构、口语表达
+归一化合并：本卡覆盖这些变体：puts it differently</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
@@ -828,17 +1199,28 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>infusion of capital</t>
+          <t>be distorted by excess</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：资本注入。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：infusion 本义是注入/泡制，引申为资金、能量或信心的注入。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济报道常用。</t>
+          <t>字面含义：被过剩扭曲；因过度而失真
+考研核心考点：distort + by 原因结构
+词汇拆解：distort = 扭曲；excess = 过度/过剩
+熟词辟义/一词多义：excess 不是 success；指过量导致问题。
+语气色彩：负面、批判</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：An infusion of capital into life sciences funded infrastructure upgrades。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：An infusion of public funding can improve rural education.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A startup may grow quickly after an infusion of capital.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济、教育投入、科技产业。</t>
+          <t>文章语境：文章说美国剑桥曾被过剩资本或过热建设扭曲。
+暗示意思/政治意味/诙谐意味：暗示太多资源也会制造泡沫和低效。
+特殊考查方式：态度题体现作者并非单纯赞美美国剑桥。
+答题技巧：注意 excess 可作名词/形容词；distorted by 后接原因。
+同义替换/错误选项信号：be warped by excess; be skewed by too much money; be damaged by overexpansion
+多场景例句：be distorted by excess；markets distorted by easy money；education distorted by excessive competition
+其他可用地方：经济、教育内卷、社会批判
+归一化合并：本卡覆盖这些变体：been distorted by excess</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
@@ -850,17 +1232,28 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>tax incentives</t>
+          <t>have an initial public offering (IPO)</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：税收激励。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：政府用减税等方式鼓励企业或个人行为。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：政策/经济常用。</t>
+          <t>字面含义：进行首次公开募股；上市
+考研核心考点：资本市场核心术语
+词汇拆解：initial = 最初的；public = 公开的；offering = 发行；IPO = initial public offering
+熟词辟义/一词多义：offering 在金融中指证券发行，不是“提供物”。
+语气色彩：正式金融语体</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：tax incentives helped attract VC funds and pharmaceutical firms。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Tax incentives can encourage companies to invest in clean energy.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Governments may use tax incentives to support innovation.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济政策、环境保护、科技创新。</t>
+          <t>文章语境：文章讨论企业是否在资本市场上市。
+暗示意思/政治意味/诙谐意味：暗示创新公司成长到一定阶段后需要公开市场融资。
+特殊考查方式：细节题会用 go public 替换。
+答题技巧：IPO = 公司第一次公开发行股票并上市。
+同义替换/错误选项信号：go public; list shares; launch an IPO
+多场景例句：have an initial public offering；go public on Nasdaq；delay an IPO during a downturn
+其他可用地方：经济、创业、资本市场
+归一化合并：本卡覆盖这些变体：have initial public offerings</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -872,17 +1265,27 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>have a presence in</t>
+          <t>overhead costs</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：在某地有业务/办公室/存在感。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：商业报道高频，比 be in 更正式。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：companies have a presence in a market/city。</t>
+          <t>字面含义：运营间接成本；日常开销
+考研核心考点：商业管理高频词
+词汇拆解：overhead = 企业固定/间接开支；costs = 成本
+熟词辟义/一词多义：overhead 不只是“头顶上方”，商业中指房租、管理、设备等间接费用。
+语气色彩：正式商业语体</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：pharma companies have a presence in Cambridge。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Many global brands have a presence in China.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Universities should have a presence in public life, not only in classrooms.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：商业、城市经济、教育社会责任。</t>
+          <t>文章语境：文章谈实验室、房租等成本压力。
+暗示意思/政治意味/诙谐意味：暗示创新企业不是只有研发问题，还有经营成本约束。
+特殊考查方式：词义题常考 overhead 的商业义。
+答题技巧：译为“间接成本/运营开销”，不要译“头顶成本”。
+同义替换/错误选项信号：operating costs; fixed costs; administrative expenses
+多场景例句：high overhead costs；cut overhead costs；overhead costs for biotech labs
+其他可用地方：职场、创业、经济生活</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
@@ -894,17 +1297,27 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>stay and scale</t>
+          <t>downturn</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：留下并扩大规模。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：scale 作动词表示扩大业务规模。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：创业/商业高频。</t>
+          <t>字面含义：经济下行；低迷期；衰退
+考研核心考点：经济周期核心词
+词汇拆解：down + turn；趋势向下
+熟词辟义/一词多义：可指市场、行业、融资环境变差。
+语气色彩：正式、负面</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Companies tend to stay and scale in American Cambridge。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Good infrastructure helps startups stay and scale.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A learner needs a method that can stay and scale with increasing difficulty.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：创业、城市发展、学习方法。</t>
+          <t>文章语境：文章提到 Kendall Square downturn 对融资和建设的影响。
+暗示意思/政治意味/诙谐意味：暗示创新生态也受经济周期影响。
+特殊考查方式：细节题可用 slump/slowdown 替换。
+答题技巧：downturn 比 recession 泛，未必是正式衰退。
+同义替换/错误选项信号：slump; slowdown; decline; recession
+多场景例句：a market downturn；a funding downturn；a downturn in biotech investment
+其他可用地方：经济、就业、创业风险</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
@@ -916,17 +1329,28 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>market cap</t>
+          <t>be left with indigestion</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：市值，market capitalisation 的缩写。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：金融/商业新闻常用。&lt;br&gt;&lt;b&gt;理解&lt;/b&gt;：公司股票总价值。</t>
+          <t>字面含义：消化不良；因过度扩张而难以消化
+考研核心考点：医学隐喻用于经济泡沫
+词汇拆解：indigestion = 消化不良；be left with = 留下/落得
+熟词辟义/一词多义：indigestion 在商业文章中可隐喻“资源过剩后的不适/后遗症”。
+语气色彩：形象、讽刺</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：two of Britain's three biggest firms by market cap。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Market cap shows how investors value a company.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A high market cap does not always mean strong social value.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济阅读、公司报道、金融常识。</t>
+          <t>文章语境：文章用它描写美国剑桥经历资本和建设过热后的不适。
+暗示意思/政治意味/诙谐意味：暗示过量资本像吃太多一样，短期繁荣后留下负担。
+特殊考查方式：修辞题/态度题：作者用幽默隐喻批评 excess。
+答题技巧：不要死译成身体胃病；按语境译“难以消化的后遗症”。
+同义替换/错误选项信号：be left with a hangover; suffer after overexpansion; struggle to digest excess
+多场景例句：be left with indigestion after a boom；a market left with a financial hangover；universities left with expansion indigestion
+其他可用地方：经济泡沫、社会反思、写作修辞
+归一化合并：本卡覆盖这些变体：was left with indigestion</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
@@ -938,17 +1362,27 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>makeshift labs</t>
+          <t>As the cranes halted, so did the funding.</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：临时改造的实验室。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：makeshift = 临时凑合的，权宜的。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：暗示条件不足、不够专业。</t>
+          <t>字面含义：吊车停了，资金也停了
+考研核心考点：as... so... 平行结构
+词汇拆解：as = 随着；cranes halted = 吊车停工；so did the funding = 资金也一样停了
+熟词辟义/一词多义：cranes 这里是建筑吊车，不是鸟。
+语气色彩：新闻体、凝练、有画面感</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：startups use office space as makeshift labs。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：创新需求增长，但基础设施跟不上。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：During emergencies, classrooms may become makeshift shelters.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A makeshift solution can help temporarily, but it cannot replace proper infrastructure.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：城市基础设施、应急管理、教育资源。</t>
+          <t>文章语境：文章用建设停摆和融资停摆形成同步对照。
+暗示意思/政治意味/诙谐意味：暗示资本热潮和地产/实验室扩建绑定，一旦降温全链条停滞。
+特殊考查方式：长难句/倒装考点：so did Y = Y also did。
+答题技巧：主干：As X halted, so did Y；译为“随着 X 停下，Y 也停了”。
+同义替换/错误选项信号：as X slowed, so did Y; when construction stopped, funding dried up
+多场景例句：As the cranes halted, so did the funding；As demand fell, so did investment；As confidence weakened, so did hiring
+其他可用地方：经济、写作句型、因果对照</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -960,17 +1394,27 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>hemmed in by</t>
+          <t>pools of capital and talent</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：被……困住/限制住。&lt;br&gt;&lt;b&gt;本义&lt;/b&gt;：hem 是衣服边，引申为被围住。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：形象，比 constrained 更有被挤压感。</t>
+          <t>字面含义：资本和人才池；大量资本与人才储备
+考研核心考点：创新生态核心搭配
+词汇拆解：pool = 水池；引申为可调用的资源集合
+熟词辟义/一词多义：pool 不只是泳池，常指人才/资金/数据集合。
+语气色彩：正式、经济管理语体</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Hemmed in by its infrastructure, Cambridge is also starved of capital。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Students hemmed in by exam pressure may lose curiosity.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Old cities are often hemmed in by limited land and transport systems.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育压力、城市发展、个人成长。</t>
+          <t>文章语境：文章说创新中心需要 pools of capital and talent。
+暗示意思/政治意味/诙谐意味：暗示创新来自资源密度和匹配效率。
+特殊考查方式：主旨题可用 concentration of resources 替换。
+答题技巧：译为“资源池/储备”，不要死译“水池”。
+同义替换/错误选项信号：reservoirs of capital and talent; concentrations of resources
+多场景例句：pools of capital and talent；a deep talent pool；a pool of research funding
+其他可用地方：教育、职场、科技创新</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
@@ -982,17 +1426,27 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>venture arm</t>
+          <t>a hedge against the Kendall Square downturn</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：风险投资部门。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：arm 不只是手臂，也指机构的分支部门。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：商业报道常用。</t>
+          <t>字面含义：对冲 Kendall Square 低迷的手段
+考研核心考点：hedge 的金融/风险管理义
+词汇拆解：hedge = 树篱；金融中指对冲/风险保护
+熟词辟义/一词多义：hedge against = protect against risk。
+语气色彩：正式金融/策略语体</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：GV, Google's venture arm。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A university may create a venture arm to support student startups.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：The charity's research arm studies public health problems.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：商业、组织结构、科技创业。</t>
+          <t>文章语境：文章说英国剑桥可成为美国 Kendall Square 低迷时的对冲选择。
+暗示意思/政治意味/诙谐意味：暗示跨地区布局可以分散风险。
+特殊考查方式：词义题可能考 hedge 的非植物义。
+答题技巧：against 后接要防范的风险。
+同义替换/错误选项信号：protection against; buffer against; insurance against
+多场景例句：a hedge against a downturn；a hedge against policy risk；overseas investment as a hedge against local weakness
+其他可用地方：经济风险、职业规划、战略布局</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
@@ -1004,17 +1458,27 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>put it differently</t>
+          <t>Atlantic alliance</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：换句话说，以另一种方式表达。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：解释、转述、推进论证常用。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：To put it differently,...</t>
+          <t>字面含义：大西洋联盟；英美/欧美合作关系
+考研核心考点：国际关系 + 科技合作表达
+词汇拆解：Atlantic = 大西洋的；alliance = 联盟
+熟词辟义/一词多义：不一定是军事联盟，也可泛指跨大西洋合作网络。
+语气色彩：正式、政治经济色彩</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Allan Bradley puts it differently 后接更尖锐的说法。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：To put it differently, discipline is freedom in the long run.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：To put it differently, technology is useful only when people use it wisely.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：作文改写、口语解释、论证推进。</t>
+          <t>文章语境：文章把两个 Cambridge 的合作放在跨大西洋创新关系中。
+暗示意思/政治意味/诙谐意味：暗示科技创新也受国际联盟和人才流动影响。
+特殊考查方式：主旨题可问文章是否强调 cooperation across the Atlantic。
+答题技巧：根据上下文决定译“跨大西洋联盟/合作”。
+同义替换/错误选项信号：transatlantic alliance; cross-Atlantic partnership; Anglo-American cooperation
+多场景例句：an Atlantic alliance in biotech；a transatlantic innovation alliance；strengthen the Atlantic alliance in research
+其他可用地方：文化交流、国际合作、科技</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
@@ -1026,17 +1490,27 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>distorted by excess</t>
+          <t>boosterish coalition</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：因过剩而被扭曲。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：批评性，常用于资本、信息、欲望、竞争过度。&lt;br&gt;&lt;b&gt;反差&lt;/b&gt;：英国缺乏，美国过剩。</t>
+          <t>字面含义：热衷鼓吹发展的联盟/联合体
+考研核心考点：态度词 boosterish
+词汇拆解：booster = 支持者/宣传者；-ish = 有……倾向的；coalition = 联盟
+熟词辟义/一词多义：boosterish 带“过分乐观、宣传味”的意味。
+语气色彩：新闻语体，略带怀疑</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：American twin has been distorted by excess。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Education can be distorted by excessive competition.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A market may be distorted by too much cheap capital.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育竞争、资本泡沫、消费主义。</t>
+          <t>文章语境：文章指推动英美剑桥合作或创新政策的一群积极倡导者。
+暗示意思/政治意味/诙谐意味：暗示他们热情高，但可能带宣传包装和利益诉求。
+特殊考查方式：态度题：boosterish 不是纯正面，带保留。
+答题技巧：译出“鼓吹/助推”，不要只译“支持”。
+同义替换/错误选项信号：promotional alliance; cheerleading coalition; pro-growth lobby
+多场景例句：a boosterish coalition；boosterish talk about innovation；a coalition of local boosters
+其他可用地方：政策宣传、城市品牌、公共伦理</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
@@ -1048,17 +1522,27 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>initial public offering (IPO)</t>
+          <t>biotech incubator</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：首次公开募股，公司上市。&lt;br&gt;&lt;b&gt;外刊常见&lt;/b&gt;：have an IPO / file for an IPO / IPO market。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：金融新闻基础词。</t>
+          <t>字面含义：生物科技孵化器
+考研核心考点：创业生态核心词
+词汇拆解：bio + tech；incubator 本义孵化器，引申为扶持初创企业的平台
+熟词辟义/一词多义：incubator 不只孵蛋设备，也指创业孵化机构。
+语气色彩：科技创业语体</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：companies began to have IPOs way too early。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：An IPO can give a company access to public capital markets.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A premature IPO may expose a weak business model.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济阅读、公司新闻、创业。</t>
+          <t>文章语境：文章提到帮助生物科技企业成长的 incubator。
+暗示意思/政治意味/诙谐意味：暗示从科研到企业需要场地、资金、导师和临床资源。
+特殊考查方式：词义题考 incubator 的创业义。
+答题技巧：译为“创业孵化器/生物科技孵化器”。
+同义替换/错误选项信号：start-up incubator; biotech accelerator; company-building platform
+多场景例句：a biotech incubator；an incubator for university spin-outs；incubate early-stage biotech firms
+其他可用地方：科技创业、教育转化、职场</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
@@ -1070,17 +1554,27 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>soared</t>
+          <t>clinical trials</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：猛增，飙升。&lt;br&gt;&lt;b&gt;本义&lt;/b&gt;：鸟向高处飞。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：新闻高频，用于价格、成本、数量、期待等急剧上升。</t>
+          <t>字面含义：临床试验
+考研核心考点：医学科技核心词
+词汇拆解：clinical = 临床的；trial = 试验
+熟词辟义/一词多义：trial 不只是审判，也指试验。
+语气色彩：正式医学语体</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Rents, overhead costs and salary expectations all soared。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Housing prices have soared in many big cities.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Students' anxiety may soar before important exams.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济、住房、教育压力、健康心理。</t>
+          <t>文章语境：文章说创新成果需要通过临床试验走向医疗应用。
+暗示意思/政治意味/诙谐意味：暗示生物科技商业化离不开医院和监管体系。
+特殊考查方式：细节题会用 human testing/medical trials 替换。
+答题技巧：不要译成“临床审判”。
+同义替换/错误选项信号：medical trials; human trials; clinical testing
+多场景例句：speed up clinical trials；run clinical trials；move a therapy into clinical trials
+其他可用地方：健康、科技、医学伦理</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
@@ -1092,17 +1586,27 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>downturn</t>
+          <t>pension reforms</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：下行期，衰退，低迷。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济金融高频。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：economic downturn / market downturn。</t>
+          <t>字面含义：养老金改革
+考研核心考点：经济政策词
+词汇拆解：pension = 养老金；reform = 改革
+熟词辟义/一词多义：pension 不等于 passion；指退休金制度。
+语气色彩：正式政策语体</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：When the downturn came, lab space was vacant and funding stopped。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：During an economic downturn, young workers need adaptable skills.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A downturn can expose weaknesses hidden during rapid growth.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济生活、职场发展、风险管理。</t>
+          <t>文章语境：文章提到养老金改革可能释放长期资本。
+暗示意思/政治意味/诙谐意味：暗示制度改革影响资本市场和创新融资。
+特殊考查方式：细节题会问什么政策能 deepen capital markets。
+答题技巧：译为“养老金改革/退休金制度改革”。
+同义替换/错误选项信号：retirement-system reform; pension-system changes
+多场景例句：pension reforms deepen capital markets；pension reforms unlock long-term capital；reform pension funds to support innovation
+其他可用地方：经济、社会保障、资本市场</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
@@ -1114,17 +1618,28 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>vacant</t>
+          <t>slashing public funding</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：空置的，空缺的。&lt;br&gt;&lt;b&gt;熟词场景&lt;/b&gt;：vacant room / vacant position / vacant lab space。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：房地产、职场、经济常用。</t>
+          <t>字面含义：大幅削减公共资金
+考研核心考点：政策变化负面搭配
+词汇拆解：slash = 猛砍/大幅削减；public funding = 公共资金
+熟词辟义/一词多义：slash 不只是“砍”，新闻中常指大幅削减预算。
+语气色彩：强负面、新闻语体</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：28% of lab space was vacant。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Many offices remain vacant after the rise of remote work.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A vacant position can create opportunities for young employees.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：职场、房地产、经济变化。</t>
+          <t>文章语境：文章说公共资金削减可能影响科研生态。
+暗示意思/政治意味/诙谐意味：暗示财政政策会直接改变创新地理。
+特殊考查方式：态度题中 slashing 显示削减幅度大。
+答题技巧：slash 后常接 budgets/costs/funding。
+同义替换/错误选项信号：cut sharply; make deep cuts to; reduce drastically
+多场景例句：slashing public funding；slash research budgets；deep cuts to university funding
+其他可用地方：教育、科研、社会责任
+归一化合并：本卡覆盖这些变体：slashing</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
@@ -1136,394 +1651,30 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>as X halted, so did Y</t>
+          <t>The geography of innovation is shifting</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：随着 X 停下，Y 也停下。&lt;br&gt;&lt;b&gt;语法&lt;/b&gt;：so did Y 是倒装，表示“Y 也如此”。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：简洁、有节奏，适合描述连锁反应。</t>
+          <t>字面含义：创新的地理格局正在变化
+考研核心考点：宏观主题句
+词汇拆解：geography = 地理分布/空间格局；innovation = 创新；shift = 转变
+熟词辟义/一词多义：geography 不只指地理课，也指资源、产业、权力的空间分布。
+语气色彩：正式、宏观判断</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：As the cranes halted, so did the funding。建筑停了，资金也停了。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：As curiosity faded, so did learning motivation.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：As public trust declined, so did cooperation.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：长难句、作文句式、因果连锁。</t>
+          <t>文章语境：文章结尾把两个 Cambridge 的关系上升为创新地理变化。
+暗示意思/政治意味/诙谐意味：暗示创新中心不再固定，资本、人才和政策会重塑版图。
+特殊考查方式：主旨题/写作主题句高价值。
+答题技巧：可作为作文句型：The geography of X is shifting。
+同义替换/错误选项信号：the map of innovation is changing; innovation is being redistributed
+多场景例句：The geography of innovation is shifting；The geography of education is shifting；The geography of work is shifting after digitalisation
+其他可用地方：科技、教育、职场、城市发展</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="53">
-      <c r="A53" t="inlineStr">
-        <is>
-          <t>larger amounts to fewer firms</t>
-        </is>
-      </c>
-      <c r="B53" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：把更大金额投给更少公司。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：资源集中，强者更强，早期弱者更难。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济/资源分配分析。</t>
-        </is>
-      </c>
-      <c r="C53" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Investors became risk-averse, giving larger amounts to fewer firms。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Scholarships sometimes give larger amounts to fewer students, leaving others unsupported.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：In a downturn, capital often goes to safer, larger firms.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育公平、经济资源、社会分配。</t>
-        </is>
-      </c>
-      <c r="D53" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="54">
-      <c r="A54" t="inlineStr">
-        <is>
-          <t>the reverse of</t>
-        </is>
-      </c>
-      <c r="B54" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：与……正好相反。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：对比论证高频。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：the reverse of the British problem。</t>
-        </is>
-      </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：美国早期公司缺资本，是英国问题的反面。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Too much control can be as harmful as too little; it is simply the reverse of the same problem.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Rural schools face the reverse of urban schools' difficulties.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：对比论证、教育、社会问题。</t>
-        </is>
-      </c>
-      <c r="D54" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="55">
-      <c r="A55" t="inlineStr">
-        <is>
-          <t>listed on the Nasdaq</t>
-        </is>
-      </c>
-      <c r="B55" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：在纳斯达克上市。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：list 不是列清单，而是股票上市。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：商业金融常用。</t>
-        </is>
-      </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Bicycle Therapeutics listed on the Nasdaq in 2019。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A company listed on a major exchange can raise more capital.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Being listed abroad may give startups access to deeper markets.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济阅读、创业、资本市场。</t>
-        </is>
-      </c>
-      <c r="D55" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="56">
-      <c r="A56" t="inlineStr">
-        <is>
-          <t>core research and development</t>
-        </is>
-      </c>
-      <c r="B56" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：核心研发。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：R&amp;D = research and development。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：科技和公司报道基础表达。</t>
-        </is>
-      </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：keep core R&amp;D at home, open office in Massachusetts。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A country should protect its core research and development capacity.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Universities contribute to core research and development in many industries.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技创新、教育、国家战略。</t>
-        </is>
-      </c>
-      <c r="D56" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="57">
-      <c r="A57" t="inlineStr">
-        <is>
-          <t>on the cheap</t>
-        </is>
-      </c>
-      <c r="B57" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：便宜地，以低成本方式。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：口语/新闻，有一点轻松甚至尖锐。&lt;br&gt;&lt;b&gt;注意&lt;/b&gt;：不是 cheap quality，而是 low cost。</t>
-        </is>
-      </c>
-      <c r="C57" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：the latter offers world-class talent on the cheap。英国提供相对便宜的世界级人才。&lt;br&gt;&lt;b&gt;暗示&lt;/b&gt;：英国人才强，但市场定价低。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Online courses can offer high-quality learning on the cheap.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Companies sometimes seek talent on the cheap in weaker labour markets.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育资源、职场、经济生活。</t>
-        </is>
-      </c>
-      <c r="D57" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="58">
-      <c r="A58" t="inlineStr">
-        <is>
-          <t>flow in the opposite direction</t>
-        </is>
-      </c>
-      <c r="B58" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：朝相反方向流动。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：资金、人才、信息、文化流动常用。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：capital/talent/data flows in the opposite direction。</t>
-        </is>
-      </c>
-      <c r="C58" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Capital is flowing in the opposite direction: US investors invest in British Cambridge。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Talent may flow in the opposite direction when policies change.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Cultural influence does not move one way; it can flow in the opposite direction.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：文化交流、人才流动、资本市场。</t>
-        </is>
-      </c>
-      <c r="D58" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" t="inlineStr">
-        <is>
-          <t>centre of excellence</t>
-        </is>
-      </c>
-      <c r="B59" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：卓越中心，优势集聚地。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：机构宣传、产业政策常用。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：某地在特定领域有顶尖能力。</t>
-        </is>
-      </c>
-      <c r="C59" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：British Cambridge is a centre of excellence。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A university can become a centre of excellence in sports science.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Cities need centres of excellence to attract investment and talent.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育、科技、城市发展、职业规划。</t>
-        </is>
-      </c>
-      <c r="D59" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" t="inlineStr">
-        <is>
-          <t>hedge against</t>
-        </is>
-      </c>
-      <c r="B60" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：对冲，防范……风险。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：hedge 不只是树篱，也指风险对冲。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：金融/风险管理常用。</t>
-        </is>
-      </c>
-      <c r="C60" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：investment in British Cambridge is a hedge against Kendall Square downturn。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Learning transferable skills is a hedge against job-market uncertainty.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Saving money can be a hedge against unexpected illness.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：职场、经济、风险管理、备考规划。</t>
-        </is>
-      </c>
-      <c r="D60" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" t="inlineStr">
-        <is>
-          <t>join up with</t>
-        </is>
-      </c>
-      <c r="B61" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：与……连接/联合起来。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：合作和网络建设常用。&lt;br&gt;&lt;b&gt;区别&lt;/b&gt;：比 cooperate with 更强调连成一体。</t>
-        </is>
-      </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：British Cambridge wants to learn from and join up with its namesake。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Schools should join up with communities to support students.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Cities can join up with universities to build innovation networks.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育合作、城市发展、文化交流。</t>
-        </is>
-      </c>
-      <c r="D61" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="62">
-      <c r="A62" t="inlineStr">
-        <is>
-          <t>modelled on</t>
-        </is>
-      </c>
-      <c r="B62" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：以……为模型，仿照……设计。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：正式，制度/建筑/项目设计常用。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：be modelled on a successful system。</t>
-        </is>
-      </c>
-      <c r="C62" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：innovation hub modelled on LabCentral。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：A new training programme can be modelled on proven methods.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Education reform should not be blindly modelled on foreign systems.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育改革、制度设计、科技园区。</t>
-        </is>
-      </c>
-      <c r="D62" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="63">
-      <c r="A63" t="inlineStr">
-        <is>
-          <t>speed up clinical trials</t>
-        </is>
-      </c>
-      <c r="B63" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：加快临床试验。&lt;br&gt;&lt;b&gt;组成&lt;/b&gt;：speed up = 加快；clinical trials = 临床试验。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：医学、药物研发常用。</t>
-        </is>
-      </c>
-      <c r="C63" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：universities and health providers work on speeding up clinical trials。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：AI may help speed up clinical trials and drug discovery.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Better cooperation can speed up public-service reform.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：健康、科技、社会责任、医学创新。</t>
-        </is>
-      </c>
-      <c r="D63" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="64">
-      <c r="A64" t="inlineStr">
-        <is>
-          <t>the squeeze on</t>
-        </is>
-      </c>
-      <c r="B64" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：……方面的紧张/压力。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：squeeze 本义挤压，引申为供应紧张或压力。&lt;br&gt;&lt;b&gt;搭配&lt;/b&gt;：the squeeze on housing / space / budgets。</t>
-        </is>
-      </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：The squeeze on lab space is easing。实验室空间紧张正在缓解。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：The squeeze on family budgets can affect children's education.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：The squeeze on urban housing makes young workers anxious.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济生活、住房、教育资源、城市发展。</t>
-        </is>
-      </c>
-      <c r="D64" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="65">
-      <c r="A65" t="inlineStr">
-        <is>
-          <t>steam ahead</t>
-        </is>
-      </c>
-      <c r="B65" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：加速推进。&lt;br&gt;&lt;b&gt;本义/诙谐&lt;/b&gt;：steam 与火车蒸汽有关，文章谈铁路项目时有轻微双关。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：新闻标题式表达。</t>
-        </is>
-      </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：railway project may finally steam ahead。谈铁路时用 steam ahead，带一点文字游戏。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：After years of delay, the education reform may finally steam ahead.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Once funding is secured, the project can steam ahead.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：项目推进、政策改革、新闻表达。</t>
-        </is>
-      </c>
-      <c r="D65" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="66">
-      <c r="A66" t="inlineStr">
-        <is>
-          <t>deepen capital markets</t>
-        </is>
-      </c>
-      <c r="B66" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：深化资本市场。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：让金融市场更成熟、更有资金深度、更能支持企业成长。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：经济政策表达。</t>
-        </is>
-      </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：Pension reforms may help Britain deepen its capital markets。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Deep capital markets can support long-term innovation.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：A country needs patient investors to deepen capital markets.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：经济、科技创业、政策阅读。</t>
-        </is>
-      </c>
-      <c r="D66" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="67">
-      <c r="A67" t="inlineStr">
-        <is>
-          <t>slashing of public funding</t>
-        </is>
-      </c>
-      <c r="B67" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：大幅削减公共经费。&lt;br&gt;&lt;b&gt;熟词辟义&lt;/b&gt;：slash 作动词/名词表示猛砍、削减。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：强烈，带批评意味。</t>
-        </is>
-      </c>
-      <c r="C67" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：America's slashing of public research funding hurt Boston-Cambridge。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：The slashing of education budgets can damage equal opportunity.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Public health suffers when funding is slashed too quickly.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：教育、科研、公共服务、社会责任。</t>
-        </is>
-      </c>
-      <c r="D67" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" t="inlineStr">
-        <is>
-          <t>geography of innovation</t>
-        </is>
-      </c>
-      <c r="B68" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：创新的地理版图。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：创新中心在哪里、如何转移、哪些地区崛起。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：外刊宏观分析表达。</t>
-        </is>
-      </c>
-      <c r="C68" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：The geography of innovation is shifting。创新中心可能从剑桥转向深圳等地。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：The geography of innovation changes when talent and capital move.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Digital tools may reshape the geography of education.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：科技、经济、城市发展、国际竞争。</t>
-        </is>
-      </c>
-      <c r="D68" t="inlineStr">
-        <is>
-          <t>外刊精读</t>
-        </is>
-      </c>
-    </row>
-    <row r="69">
-      <c r="A69" t="inlineStr">
-        <is>
-          <t>draw A closer</t>
-        </is>
-      </c>
-      <c r="B69" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;核心义&lt;/b&gt;：使 A 更加靠近/更紧密。&lt;br&gt;&lt;b&gt;引申义&lt;/b&gt;：外部压力促成合作。&lt;br&gt;&lt;b&gt;语气&lt;/b&gt;：国际关系、组织合作常用。</t>
-        </is>
-      </c>
-      <c r="C69" t="inlineStr">
-        <is>
-          <t>&lt;b&gt;文章语境&lt;/b&gt;：competition from China may draw the Cambridges closer still。&lt;br&gt;&lt;b&gt;例句1&lt;/b&gt;：Shared challenges can draw different communities closer.&lt;br&gt;&lt;b&gt;例句2&lt;/b&gt;：Global problems should draw countries closer, not push them apart.&lt;br&gt;&lt;b&gt;可用场景&lt;/b&gt;：文化交流、国际合作、社会责任。</t>
-        </is>
-      </c>
-      <c r="D69" t="inlineStr">
         <is>
           <t>外刊精读</t>
         </is>
@@ -1616,7 +1767,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>英语::外刊精读</t>
+          <t>考研英语::外刊精读</t>
         </is>
       </c>
     </row>

</xml_diff>